<commit_message>
Move validation to header row. Temp hard code 1230 to be settlement
</commit_message>
<xml_diff>
--- a/instruction_data/templates/dec_final/Nature.xlsx
+++ b/instruction_data/templates/dec_final/Nature.xlsx
@@ -8,16 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyle/projects/onesky_financial_agent/instruction_data/templates/dec_final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{69BCA014-658D-C346-82E0-E14537F8B581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{633EE9D9-E805-5A41-8C3B-B2529A2D5C66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2160" yWindow="980" windowWidth="27640" windowHeight="15520" xr2:uid="{9EF6B62F-ECF7-2B4A-949E-AD2495D5CCF8}"/>
+    <workbookView xWindow="1160" yWindow="980" windowWidth="27640" windowHeight="15520" xr2:uid="{9EF6B62F-ECF7-2B4A-949E-AD2495D5CCF8}"/>
   </bookViews>
   <sheets>
     <sheet name="Lookup1_AcctList" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Lookup1_AcctList!$A$2:$H$84</definedName>
     <definedName name="CHActCashBalance">#REF!</definedName>
@@ -500,40 +497,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Transaction List with Splits"/>
-      <sheetName val="BS manual mapping"/>
-      <sheetName val="Lookup2_province"/>
-      <sheetName val="Lookup3_Staff &amp; allocation"/>
-      <sheetName val="salary allocation-v2"/>
-      <sheetName val="PIT+SI payment"/>
-      <sheetName val="PIT+SI payment (2)"/>
-      <sheetName val="30 Bank VN Vietnam (VND)"/>
-      <sheetName val="29 Bank VN Vietnam (USD)"/>
-      <sheetName val="34 Bank VN Vietnam (VND)"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1520,7 +1483,7 @@
         <v>6</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84" spans="1:2" ht="14" x14ac:dyDescent="0.15">

</xml_diff>